<commit_message>
Fix #NAME? errors: replace dot-notation functions with compatible equivalents in 03_Probability_Distributions.xlsx
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-12/03_Probability_Distributions.xlsx
+++ b/rFLA300/chapter-12/03_Probability_Distributions.xlsx
@@ -584,6 +584,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -632,6 +633,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
@@ -676,7 +678,7 @@
         </is>
       </c>
       <c r="D9" s="11">
-        <f>NORM.DIST(40000,B5,B6,TRUE)</f>
+        <f>NORMDIST(40000,B5,B6,TRUE)</f>
         <v/>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -702,7 +704,7 @@
         </is>
       </c>
       <c r="D10" s="11">
-        <f>1-NORM.DIST(60000,B5,B6,TRUE)</f>
+        <f>1-NORMDIST(60000,B5,B6,TRUE)</f>
         <v/>
       </c>
       <c r="E10" s="14" t="inlineStr">
@@ -728,7 +730,7 @@
         </is>
       </c>
       <c r="D11" s="11">
-        <f>NORM.DIST(58000,B5,B6,TRUE)-NORM.DIST(42000,B5,B6,TRUE)</f>
+        <f>NORMDIST(58000,B5,B6,TRUE)-NORMDIST(42000,B5,B6,TRUE)</f>
         <v/>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -754,7 +756,7 @@
         </is>
       </c>
       <c r="D12" s="15">
-        <f>NORM.INV(0.95,B5,B6)</f>
+        <f>NORMINV(0.95,B5,B6)</f>
         <v/>
       </c>
       <c r="E12" s="14" t="inlineStr">
@@ -780,7 +782,7 @@
         </is>
       </c>
       <c r="D13" s="15">
-        <f>NORM.INV(0.25,B5,B6)</f>
+        <f>NORMINV(0.25,B5,B6)</f>
         <v/>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -789,6 +791,8 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
@@ -823,11 +827,11 @@
         <v>-3</v>
       </c>
       <c r="B18" s="18">
-        <f>NORM.DIST(-3,0,1,TRUE)</f>
+        <f>NORMDIST(-3,0,1,TRUE)</f>
         <v/>
       </c>
       <c r="C18" s="18">
-        <f>NORM.DIST(-3,0,1,FALSE)</f>
+        <f>NORMDIST(-3,0,1,FALSE)</f>
         <v/>
       </c>
       <c r="D18" s="19" t="inlineStr">
@@ -841,11 +845,11 @@
         <v>-2.5</v>
       </c>
       <c r="B19" s="18">
-        <f>NORM.DIST(-2.5,0,1,TRUE)</f>
+        <f>NORMDIST(-2.5,0,1,TRUE)</f>
         <v/>
       </c>
       <c r="C19" s="18">
-        <f>NORM.DIST(-2.5,0,1,FALSE)</f>
+        <f>NORMDIST(-2.5,0,1,FALSE)</f>
         <v/>
       </c>
       <c r="D19" s="21" t="inlineStr"/>
@@ -855,11 +859,11 @@
         <v>-2</v>
       </c>
       <c r="B20" s="18">
-        <f>NORM.DIST(-2,0,1,TRUE)</f>
+        <f>NORMDIST(-2,0,1,TRUE)</f>
         <v/>
       </c>
       <c r="C20" s="18">
-        <f>NORM.DIST(-2,0,1,FALSE)</f>
+        <f>NORMDIST(-2,0,1,FALSE)</f>
         <v/>
       </c>
       <c r="D20" s="19" t="inlineStr">
@@ -873,11 +877,11 @@
         <v>-1.5</v>
       </c>
       <c r="B21" s="18">
-        <f>NORM.DIST(-1.5,0,1,TRUE)</f>
+        <f>NORMDIST(-1.5,0,1,TRUE)</f>
         <v/>
       </c>
       <c r="C21" s="18">
-        <f>NORM.DIST(-1.5,0,1,FALSE)</f>
+        <f>NORMDIST(-1.5,0,1,FALSE)</f>
         <v/>
       </c>
       <c r="D21" s="21" t="inlineStr"/>
@@ -887,11 +891,11 @@
         <v>-1</v>
       </c>
       <c r="B22" s="18">
-        <f>NORM.DIST(-1,0,1,TRUE)</f>
+        <f>NORMDIST(-1,0,1,TRUE)</f>
         <v/>
       </c>
       <c r="C22" s="18">
-        <f>NORM.DIST(-1,0,1,FALSE)</f>
+        <f>NORMDIST(-1,0,1,FALSE)</f>
         <v/>
       </c>
       <c r="D22" s="19" t="inlineStr">
@@ -905,11 +909,11 @@
         <v>-0.5</v>
       </c>
       <c r="B23" s="18">
-        <f>NORM.DIST(-0.5,0,1,TRUE)</f>
+        <f>NORMDIST(-0.5,0,1,TRUE)</f>
         <v/>
       </c>
       <c r="C23" s="18">
-        <f>NORM.DIST(-0.5,0,1,FALSE)</f>
+        <f>NORMDIST(-0.5,0,1,FALSE)</f>
         <v/>
       </c>
       <c r="D23" s="21" t="inlineStr"/>
@@ -919,11 +923,11 @@
         <v>0</v>
       </c>
       <c r="B24" s="18">
-        <f>NORM.DIST(0,0,1,TRUE)</f>
+        <f>NORMDIST(0,0,1,TRUE)</f>
         <v/>
       </c>
       <c r="C24" s="18">
-        <f>NORM.DIST(0,0,1,FALSE)</f>
+        <f>NORMDIST(0,0,1,FALSE)</f>
         <v/>
       </c>
       <c r="D24" s="19" t="inlineStr">
@@ -937,11 +941,11 @@
         <v>0.5</v>
       </c>
       <c r="B25" s="18">
-        <f>NORM.DIST(0.5,0,1,TRUE)</f>
+        <f>NORMDIST(0.5,0,1,TRUE)</f>
         <v/>
       </c>
       <c r="C25" s="18">
-        <f>NORM.DIST(0.5,0,1,FALSE)</f>
+        <f>NORMDIST(0.5,0,1,FALSE)</f>
         <v/>
       </c>
       <c r="D25" s="21" t="inlineStr"/>
@@ -951,11 +955,11 @@
         <v>1</v>
       </c>
       <c r="B26" s="18">
-        <f>NORM.DIST(1,0,1,TRUE)</f>
+        <f>NORMDIST(1,0,1,TRUE)</f>
         <v/>
       </c>
       <c r="C26" s="18">
-        <f>NORM.DIST(1,0,1,FALSE)</f>
+        <f>NORMDIST(1,0,1,FALSE)</f>
         <v/>
       </c>
       <c r="D26" s="19" t="inlineStr">
@@ -969,11 +973,11 @@
         <v>1.5</v>
       </c>
       <c r="B27" s="18">
-        <f>NORM.DIST(1.5,0,1,TRUE)</f>
+        <f>NORMDIST(1.5,0,1,TRUE)</f>
         <v/>
       </c>
       <c r="C27" s="18">
-        <f>NORM.DIST(1.5,0,1,FALSE)</f>
+        <f>NORMDIST(1.5,0,1,FALSE)</f>
         <v/>
       </c>
       <c r="D27" s="21" t="inlineStr"/>
@@ -983,11 +987,11 @@
         <v>2</v>
       </c>
       <c r="B28" s="18">
-        <f>NORM.DIST(2,0,1,TRUE)</f>
+        <f>NORMDIST(2,0,1,TRUE)</f>
         <v/>
       </c>
       <c r="C28" s="18">
-        <f>NORM.DIST(2,0,1,FALSE)</f>
+        <f>NORMDIST(2,0,1,FALSE)</f>
         <v/>
       </c>
       <c r="D28" s="19" t="inlineStr">
@@ -1001,11 +1005,11 @@
         <v>2.5</v>
       </c>
       <c r="B29" s="18">
-        <f>NORM.DIST(2.5,0,1,TRUE)</f>
+        <f>NORMDIST(2.5,0,1,TRUE)</f>
         <v/>
       </c>
       <c r="C29" s="18">
-        <f>NORM.DIST(2.5,0,1,FALSE)</f>
+        <f>NORMDIST(2.5,0,1,FALSE)</f>
         <v/>
       </c>
       <c r="D29" s="21" t="inlineStr"/>
@@ -1015,11 +1019,11 @@
         <v>3</v>
       </c>
       <c r="B30" s="18">
-        <f>NORM.DIST(3,0,1,TRUE)</f>
+        <f>NORMDIST(3,0,1,TRUE)</f>
         <v/>
       </c>
       <c r="C30" s="18">
-        <f>NORM.DIST(3,0,1,FALSE)</f>
+        <f>NORMDIST(3,0,1,FALSE)</f>
         <v/>
       </c>
       <c r="D30" s="19" t="inlineStr">
@@ -1028,6 +1032,8 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="22" t="inlineStr">
         <is>
@@ -1077,6 +1083,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1125,6 +1132,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
@@ -1167,7 +1175,7 @@
         </is>
       </c>
       <c r="D9" s="11">
-        <f>BINOM.DIST(0,B5,B6,FALSE)</f>
+        <f>BINOMDIST(0,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -1191,7 +1199,7 @@
         </is>
       </c>
       <c r="D10" s="11">
-        <f>BINOM.DIST(2,B5,B6,FALSE)</f>
+        <f>BINOMDIST(2,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="E10" s="14" t="inlineStr">
@@ -1215,7 +1223,7 @@
         </is>
       </c>
       <c r="D11" s="11">
-        <f>BINOM.DIST(3,B5,B6,TRUE)</f>
+        <f>BINOMDIST(3,B5,B6,TRUE)</f>
         <v/>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -1241,7 +1249,7 @@
         </is>
       </c>
       <c r="D12" s="11">
-        <f>1-BINOM.DIST(2,B5,B6,TRUE)</f>
+        <f>1-BINOMDIST(2,B5,B6,TRUE)</f>
         <v/>
       </c>
       <c r="E12" s="14" t="inlineStr">
@@ -1267,7 +1275,7 @@
         </is>
       </c>
       <c r="D13" s="11">
-        <f>BINOM.DIST(4,B5,B6,TRUE)-BINOM.DIST(0,B5,B6,TRUE)</f>
+        <f>BINOMDIST(4,B5,B6,TRUE)-BINOMDIST(0,B5,B6,TRUE)</f>
         <v/>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -1276,6 +1284,8 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
@@ -1305,11 +1315,11 @@
         <v>0</v>
       </c>
       <c r="B18" s="25">
-        <f>BINOM.DIST(0,B5,B6,FALSE)</f>
+        <f>BINOMDIST(0,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C18" s="25">
-        <f>BINOM.DIST(0,B5,B6,TRUE)</f>
+        <f>BINOMDIST(0,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1318,11 +1328,11 @@
         <v>1</v>
       </c>
       <c r="B19" s="25">
-        <f>BINOM.DIST(1,B5,B6,FALSE)</f>
+        <f>BINOMDIST(1,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C19" s="25">
-        <f>BINOM.DIST(1,B5,B6,TRUE)</f>
+        <f>BINOMDIST(1,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1331,11 +1341,11 @@
         <v>2</v>
       </c>
       <c r="B20" s="25">
-        <f>BINOM.DIST(2,B5,B6,FALSE)</f>
+        <f>BINOMDIST(2,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C20" s="25">
-        <f>BINOM.DIST(2,B5,B6,TRUE)</f>
+        <f>BINOMDIST(2,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1344,11 +1354,11 @@
         <v>3</v>
       </c>
       <c r="B21" s="25">
-        <f>BINOM.DIST(3,B5,B6,FALSE)</f>
+        <f>BINOMDIST(3,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C21" s="25">
-        <f>BINOM.DIST(3,B5,B6,TRUE)</f>
+        <f>BINOMDIST(3,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1357,11 +1367,11 @@
         <v>4</v>
       </c>
       <c r="B22" s="25">
-        <f>BINOM.DIST(4,B5,B6,FALSE)</f>
+        <f>BINOMDIST(4,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C22" s="25">
-        <f>BINOM.DIST(4,B5,B6,TRUE)</f>
+        <f>BINOMDIST(4,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1370,11 +1380,11 @@
         <v>5</v>
       </c>
       <c r="B23" s="25">
-        <f>BINOM.DIST(5,B5,B6,FALSE)</f>
+        <f>BINOMDIST(5,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C23" s="25">
-        <f>BINOM.DIST(5,B5,B6,TRUE)</f>
+        <f>BINOMDIST(5,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1383,11 +1393,11 @@
         <v>6</v>
       </c>
       <c r="B24" s="25">
-        <f>BINOM.DIST(6,B5,B6,FALSE)</f>
+        <f>BINOMDIST(6,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C24" s="25">
-        <f>BINOM.DIST(6,B5,B6,TRUE)</f>
+        <f>BINOMDIST(6,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1396,11 +1406,11 @@
         <v>7</v>
       </c>
       <c r="B25" s="25">
-        <f>BINOM.DIST(7,B5,B6,FALSE)</f>
+        <f>BINOMDIST(7,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C25" s="25">
-        <f>BINOM.DIST(7,B5,B6,TRUE)</f>
+        <f>BINOMDIST(7,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1409,11 +1419,11 @@
         <v>8</v>
       </c>
       <c r="B26" s="25">
-        <f>BINOM.DIST(8,B5,B6,FALSE)</f>
+        <f>BINOMDIST(8,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C26" s="25">
-        <f>BINOM.DIST(8,B5,B6,TRUE)</f>
+        <f>BINOMDIST(8,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1422,11 +1432,11 @@
         <v>9</v>
       </c>
       <c r="B27" s="25">
-        <f>BINOM.DIST(9,B5,B6,FALSE)</f>
+        <f>BINOMDIST(9,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C27" s="25">
-        <f>BINOM.DIST(9,B5,B6,TRUE)</f>
+        <f>BINOMDIST(9,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1435,11 +1445,11 @@
         <v>10</v>
       </c>
       <c r="B28" s="25">
-        <f>BINOM.DIST(10,B5,B6,FALSE)</f>
+        <f>BINOMDIST(10,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C28" s="25">
-        <f>BINOM.DIST(10,B5,B6,TRUE)</f>
+        <f>BINOMDIST(10,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1448,11 +1458,11 @@
         <v>11</v>
       </c>
       <c r="B29" s="25">
-        <f>BINOM.DIST(11,B5,B6,FALSE)</f>
+        <f>BINOMDIST(11,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C29" s="25">
-        <f>BINOM.DIST(11,B5,B6,TRUE)</f>
+        <f>BINOMDIST(11,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1461,11 +1471,11 @@
         <v>12</v>
       </c>
       <c r="B30" s="25">
-        <f>BINOM.DIST(12,B5,B6,FALSE)</f>
+        <f>BINOMDIST(12,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C30" s="25">
-        <f>BINOM.DIST(12,B5,B6,TRUE)</f>
+        <f>BINOMDIST(12,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1474,11 +1484,11 @@
         <v>13</v>
       </c>
       <c r="B31" s="25">
-        <f>BINOM.DIST(13,B5,B6,FALSE)</f>
+        <f>BINOMDIST(13,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C31" s="25">
-        <f>BINOM.DIST(13,B5,B6,TRUE)</f>
+        <f>BINOMDIST(13,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1487,11 +1497,11 @@
         <v>14</v>
       </c>
       <c r="B32" s="25">
-        <f>BINOM.DIST(14,B5,B6,FALSE)</f>
+        <f>BINOMDIST(14,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C32" s="25">
-        <f>BINOM.DIST(14,B5,B6,TRUE)</f>
+        <f>BINOMDIST(14,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1500,11 +1510,11 @@
         <v>15</v>
       </c>
       <c r="B33" s="25">
-        <f>BINOM.DIST(15,B5,B6,FALSE)</f>
+        <f>BINOMDIST(15,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C33" s="25">
-        <f>BINOM.DIST(15,B5,B6,TRUE)</f>
+        <f>BINOMDIST(15,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1513,11 +1523,11 @@
         <v>16</v>
       </c>
       <c r="B34" s="25">
-        <f>BINOM.DIST(16,B5,B6,FALSE)</f>
+        <f>BINOMDIST(16,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C34" s="25">
-        <f>BINOM.DIST(16,B5,B6,TRUE)</f>
+        <f>BINOMDIST(16,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1526,11 +1536,11 @@
         <v>17</v>
       </c>
       <c r="B35" s="25">
-        <f>BINOM.DIST(17,B5,B6,FALSE)</f>
+        <f>BINOMDIST(17,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C35" s="25">
-        <f>BINOM.DIST(17,B5,B6,TRUE)</f>
+        <f>BINOMDIST(17,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1539,11 +1549,11 @@
         <v>18</v>
       </c>
       <c r="B36" s="25">
-        <f>BINOM.DIST(18,B5,B6,FALSE)</f>
+        <f>BINOMDIST(18,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C36" s="25">
-        <f>BINOM.DIST(18,B5,B6,TRUE)</f>
+        <f>BINOMDIST(18,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1552,11 +1562,11 @@
         <v>19</v>
       </c>
       <c r="B37" s="25">
-        <f>BINOM.DIST(19,B5,B6,FALSE)</f>
+        <f>BINOMDIST(19,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C37" s="25">
-        <f>BINOM.DIST(19,B5,B6,TRUE)</f>
+        <f>BINOMDIST(19,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1565,11 +1575,11 @@
         <v>20</v>
       </c>
       <c r="B38" s="25">
-        <f>BINOM.DIST(20,B5,B6,FALSE)</f>
+        <f>BINOMDIST(20,B5,B6,FALSE)</f>
         <v/>
       </c>
       <c r="C38" s="25">
-        <f>BINOM.DIST(20,B5,B6,TRUE)</f>
+        <f>BINOMDIST(20,B5,B6,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1614,6 +1624,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1647,6 +1658,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
@@ -1689,7 +1701,7 @@
         </is>
       </c>
       <c r="D8" s="11">
-        <f>POISSON.DIST(10,B5,FALSE)</f>
+        <f>POISSON(10,B5,FALSE)</f>
         <v/>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -1713,7 +1725,7 @@
         </is>
       </c>
       <c r="D9" s="11">
-        <f>POISSON.DIST(7,B5,TRUE)</f>
+        <f>POISSON(7,B5,TRUE)</f>
         <v/>
       </c>
       <c r="E9" s="14" t="inlineStr">
@@ -1739,7 +1751,7 @@
         </is>
       </c>
       <c r="D10" s="11">
-        <f>1-POISSON.DIST(15,B5,TRUE)</f>
+        <f>1-POISSON(15,B5,TRUE)</f>
         <v/>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -1765,7 +1777,7 @@
         </is>
       </c>
       <c r="D11" s="11">
-        <f>POISSON.DIST(14,B5,TRUE)-POISSON.DIST(9,B5,TRUE)</f>
+        <f>POISSON(14,B5,TRUE)-POISSON(9,B5,TRUE)</f>
         <v/>
       </c>
       <c r="E11" s="14" t="inlineStr">
@@ -1789,7 +1801,7 @@
         </is>
       </c>
       <c r="D12" s="11">
-        <f>POISSON.DIST(0,B5,FALSE)</f>
+        <f>POISSON(0,B5,FALSE)</f>
         <v/>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1798,6 +1810,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
@@ -1827,11 +1840,11 @@
         <v>0</v>
       </c>
       <c r="B16" s="25">
-        <f>POISSON.DIST(0,B5,FALSE)</f>
+        <f>POISSON(0,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C16" s="25">
-        <f>POISSON.DIST(0,B5,TRUE)</f>
+        <f>POISSON(0,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1840,11 +1853,11 @@
         <v>1</v>
       </c>
       <c r="B17" s="25">
-        <f>POISSON.DIST(1,B5,FALSE)</f>
+        <f>POISSON(1,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C17" s="25">
-        <f>POISSON.DIST(1,B5,TRUE)</f>
+        <f>POISSON(1,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1853,11 +1866,11 @@
         <v>2</v>
       </c>
       <c r="B18" s="25">
-        <f>POISSON.DIST(2,B5,FALSE)</f>
+        <f>POISSON(2,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C18" s="25">
-        <f>POISSON.DIST(2,B5,TRUE)</f>
+        <f>POISSON(2,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1866,11 +1879,11 @@
         <v>3</v>
       </c>
       <c r="B19" s="25">
-        <f>POISSON.DIST(3,B5,FALSE)</f>
+        <f>POISSON(3,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C19" s="25">
-        <f>POISSON.DIST(3,B5,TRUE)</f>
+        <f>POISSON(3,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1879,11 +1892,11 @@
         <v>4</v>
       </c>
       <c r="B20" s="25">
-        <f>POISSON.DIST(4,B5,FALSE)</f>
+        <f>POISSON(4,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C20" s="25">
-        <f>POISSON.DIST(4,B5,TRUE)</f>
+        <f>POISSON(4,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1892,11 +1905,11 @@
         <v>5</v>
       </c>
       <c r="B21" s="25">
-        <f>POISSON.DIST(5,B5,FALSE)</f>
+        <f>POISSON(5,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C21" s="25">
-        <f>POISSON.DIST(5,B5,TRUE)</f>
+        <f>POISSON(5,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1905,11 +1918,11 @@
         <v>6</v>
       </c>
       <c r="B22" s="25">
-        <f>POISSON.DIST(6,B5,FALSE)</f>
+        <f>POISSON(6,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C22" s="25">
-        <f>POISSON.DIST(6,B5,TRUE)</f>
+        <f>POISSON(6,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1918,11 +1931,11 @@
         <v>7</v>
       </c>
       <c r="B23" s="25">
-        <f>POISSON.DIST(7,B5,FALSE)</f>
+        <f>POISSON(7,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C23" s="25">
-        <f>POISSON.DIST(7,B5,TRUE)</f>
+        <f>POISSON(7,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1931,11 +1944,11 @@
         <v>8</v>
       </c>
       <c r="B24" s="25">
-        <f>POISSON.DIST(8,B5,FALSE)</f>
+        <f>POISSON(8,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C24" s="25">
-        <f>POISSON.DIST(8,B5,TRUE)</f>
+        <f>POISSON(8,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1944,11 +1957,11 @@
         <v>9</v>
       </c>
       <c r="B25" s="25">
-        <f>POISSON.DIST(9,B5,FALSE)</f>
+        <f>POISSON(9,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C25" s="25">
-        <f>POISSON.DIST(9,B5,TRUE)</f>
+        <f>POISSON(9,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1957,11 +1970,11 @@
         <v>10</v>
       </c>
       <c r="B26" s="25">
-        <f>POISSON.DIST(10,B5,FALSE)</f>
+        <f>POISSON(10,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C26" s="25">
-        <f>POISSON.DIST(10,B5,TRUE)</f>
+        <f>POISSON(10,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1970,11 +1983,11 @@
         <v>11</v>
       </c>
       <c r="B27" s="25">
-        <f>POISSON.DIST(11,B5,FALSE)</f>
+        <f>POISSON(11,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C27" s="25">
-        <f>POISSON.DIST(11,B5,TRUE)</f>
+        <f>POISSON(11,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1983,11 +1996,11 @@
         <v>12</v>
       </c>
       <c r="B28" s="25">
-        <f>POISSON.DIST(12,B5,FALSE)</f>
+        <f>POISSON(12,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C28" s="25">
-        <f>POISSON.DIST(12,B5,TRUE)</f>
+        <f>POISSON(12,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -1996,11 +2009,11 @@
         <v>13</v>
       </c>
       <c r="B29" s="25">
-        <f>POISSON.DIST(13,B5,FALSE)</f>
+        <f>POISSON(13,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C29" s="25">
-        <f>POISSON.DIST(13,B5,TRUE)</f>
+        <f>POISSON(13,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -2009,11 +2022,11 @@
         <v>14</v>
       </c>
       <c r="B30" s="25">
-        <f>POISSON.DIST(14,B5,FALSE)</f>
+        <f>POISSON(14,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C30" s="25">
-        <f>POISSON.DIST(14,B5,TRUE)</f>
+        <f>POISSON(14,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -2022,11 +2035,11 @@
         <v>15</v>
       </c>
       <c r="B31" s="25">
-        <f>POISSON.DIST(15,B5,FALSE)</f>
+        <f>POISSON(15,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C31" s="25">
-        <f>POISSON.DIST(15,B5,TRUE)</f>
+        <f>POISSON(15,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -2035,11 +2048,11 @@
         <v>16</v>
       </c>
       <c r="B32" s="25">
-        <f>POISSON.DIST(16,B5,FALSE)</f>
+        <f>POISSON(16,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C32" s="25">
-        <f>POISSON.DIST(16,B5,TRUE)</f>
+        <f>POISSON(16,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -2048,11 +2061,11 @@
         <v>17</v>
       </c>
       <c r="B33" s="25">
-        <f>POISSON.DIST(17,B5,FALSE)</f>
+        <f>POISSON(17,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C33" s="25">
-        <f>POISSON.DIST(17,B5,TRUE)</f>
+        <f>POISSON(17,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -2061,11 +2074,11 @@
         <v>18</v>
       </c>
       <c r="B34" s="25">
-        <f>POISSON.DIST(18,B5,FALSE)</f>
+        <f>POISSON(18,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C34" s="25">
-        <f>POISSON.DIST(18,B5,TRUE)</f>
+        <f>POISSON(18,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -2074,11 +2087,11 @@
         <v>19</v>
       </c>
       <c r="B35" s="25">
-        <f>POISSON.DIST(19,B5,FALSE)</f>
+        <f>POISSON(19,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C35" s="25">
-        <f>POISSON.DIST(19,B5,TRUE)</f>
+        <f>POISSON(19,B5,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -2087,11 +2100,11 @@
         <v>20</v>
       </c>
       <c r="B36" s="25">
-        <f>POISSON.DIST(20,B5,FALSE)</f>
+        <f>POISSON(20,B5,FALSE)</f>
         <v/>
       </c>
       <c r="C36" s="25">
-        <f>POISSON.DIST(20,B5,TRUE)</f>
+        <f>POISSON(20,B5,TRUE)</f>
         <v/>
       </c>
     </row>

</xml_diff>